<commit_message>
Harden XLSX upload validation and admin-only upload/import
</commit_message>
<xml_diff>
--- a/templates/resit-template.xlsx
+++ b/templates/resit-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Project\crud\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0B310476C7BE641D9773D53CF56FA391272E6D8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E5DF549-5C58-4343-9659-127006091DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -303,7 +303,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -313,30 +313,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -411,6 +387,24 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -747,90 +741,90 @@
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="36"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
     </row>
     <row r="8" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="L8" s="6"/>
     </row>
     <row r="9" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="39"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
       <c r="L9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M9" s="38"/>
-      <c r="N9" s="38"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="30"/>
     </row>
     <row r="10" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
       <c r="L10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M10" s="38"/>
-      <c r="N10" s="38"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
     </row>
     <row r="11" spans="2:14" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
@@ -847,72 +841,72 @@
       <c r="M12" s="2"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="37"/>
-      <c r="L13" s="37"/>
-      <c r="M13" s="37"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
+      <c r="K13" s="29"/>
+      <c r="L13" s="29"/>
+      <c r="M13" s="29"/>
     </row>
     <row r="14" spans="2:14" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37"/>
-      <c r="K14" s="37"/>
-      <c r="L14" s="37"/>
-      <c r="M14" s="37"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="29"/>
+      <c r="L14" s="29"/>
+      <c r="M14" s="29"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="29" t="s">
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="I16" s="33"/>
-      <c r="J16" s="29" t="s">
+      <c r="I16" s="25"/>
+      <c r="J16" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="K16" s="30"/>
-      <c r="L16" s="33"/>
-      <c r="M16" s="30" t="s">
+      <c r="K16" s="22"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="N16" s="33"/>
+      <c r="N16" s="25"/>
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="31"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="32"/>
-      <c r="L17" s="34"/>
-      <c r="M17" s="32"/>
-      <c r="N17" s="34"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="24"/>
+      <c r="N17" s="26"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
@@ -939,52 +933,52 @@
       <c r="N20" s="5"/>
     </row>
     <row r="21" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="35"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="16"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="11">
+      <c r="B21" s="27"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="36">
         <f>SUM(H21*J21)</f>
         <v>0</v>
       </c>
-      <c r="N21" s="12"/>
+      <c r="N21" s="37"/>
     </row>
     <row r="22" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="35"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="12"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="36"/>
+      <c r="N22" s="37"/>
     </row>
     <row r="23" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="35"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="12"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="36"/>
+      <c r="N23" s="37"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="4"/>
@@ -1003,19 +997,19 @@
       <c r="N25" s="5"/>
     </row>
     <row r="26" spans="2:14" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="27"/>
+      <c r="C26" s="19"/>
       <c r="H26" s="4"/>
       <c r="I26" s="5"/>
       <c r="J26" s="4"/>
       <c r="L26" s="5"/>
-      <c r="M26" s="13">
+      <c r="M26" s="36">
         <f>-SUM(H26:L26)</f>
         <v>0</v>
       </c>
-      <c r="N26" s="14"/>
+      <c r="N26" s="37"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="4"/>
@@ -1066,39 +1060,39 @@
       <c r="N32" s="5"/>
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="22"/>
-      <c r="M33" s="7">
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="13"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="32">
         <f>SUM(M18:N32)</f>
         <v>0</v>
       </c>
-      <c r="N33" s="8"/>
+      <c r="N33" s="33"/>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B34" s="23"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="9"/>
-      <c r="N34" s="10"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="16"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="17"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="35"/>
     </row>
     <row r="37" spans="2:16" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B37" s="6" t="s">
@@ -1106,23 +1100,23 @@
       </c>
     </row>
     <row r="40" spans="2:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B40" s="28" t="s">
+      <c r="B40" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="28"/>
-      <c r="K40" s="28"/>
-      <c r="L40" s="28"/>
-      <c r="M40" s="28"/>
-      <c r="N40" s="28"/>
-      <c r="O40" s="28"/>
-      <c r="P40" s="28"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="20"/>
+      <c r="N40" s="20"/>
+      <c r="O40" s="20"/>
+      <c r="P40" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>

<commit_message>
Fix: tambah mapping M21 (subtotal) dalam export resit
</commit_message>
<xml_diff>
--- a/templates/resit-template.xlsx
+++ b/templates/resit-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Project\crud\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E5DF549-5C58-4343-9659-127006091DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C98B73-B415-46A9-A8D5-ABDD846424C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -313,14 +313,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -352,59 +397,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -741,90 +741,90 @@
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="L8" s="6"/>
     </row>
     <row r="9" spans="2:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
       <c r="L9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
     </row>
     <row r="10" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
       <c r="L10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
     </row>
     <row r="11" spans="2:14" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
@@ -841,72 +841,72 @@
       <c r="M12" s="2"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29"/>
-      <c r="K13" s="29"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
     </row>
     <row r="14" spans="2:14" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="29"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="29"/>
-      <c r="M14" s="29"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="21" t="s">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I16" s="25"/>
-      <c r="J16" s="21" t="s">
+      <c r="I16" s="16"/>
+      <c r="J16" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="K16" s="22"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="22" t="s">
+      <c r="K16" s="13"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="N16" s="25"/>
+      <c r="N16" s="16"/>
     </row>
     <row r="17" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="26"/>
-      <c r="M17" s="24"/>
-      <c r="N17" s="26"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="17"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
@@ -933,52 +933,54 @@
       <c r="N20" s="5"/>
     </row>
     <row r="21" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="27"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="36">
+      <c r="B21" s="18"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="35">
+        <v>0</v>
+      </c>
+      <c r="K21" s="36"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="23">
         <f>SUM(H21*J21)</f>
         <v>0</v>
       </c>
-      <c r="N21" s="37"/>
+      <c r="N21" s="24"/>
     </row>
     <row r="22" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="27"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="36"/>
-      <c r="N22" s="37"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="35"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="37"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="24"/>
     </row>
     <row r="23" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="27"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="37"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="35"/>
+      <c r="K23" s="36"/>
+      <c r="L23" s="37"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="24"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="4"/>
@@ -997,19 +999,19 @@
       <c r="N25" s="5"/>
     </row>
     <row r="26" spans="2:14" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="19"/>
+      <c r="C26" s="34"/>
       <c r="H26" s="4"/>
       <c r="I26" s="5"/>
       <c r="J26" s="4"/>
       <c r="L26" s="5"/>
-      <c r="M26" s="36">
+      <c r="M26" s="23">
         <f>-SUM(H26:L26)</f>
         <v>0</v>
       </c>
-      <c r="N26" s="37"/>
+      <c r="N26" s="24"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="4"/>
@@ -1060,39 +1062,39 @@
       <c r="N32" s="5"/>
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="32">
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="28"/>
+      <c r="L33" s="29"/>
+      <c r="M33" s="19">
         <f>SUM(M18:N32)</f>
         <v>0</v>
       </c>
-      <c r="N33" s="33"/>
+      <c r="N33" s="20"/>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B34" s="15"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="17"/>
-      <c r="M34" s="34"/>
-      <c r="N34" s="35"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="31"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="21"/>
+      <c r="N34" s="22"/>
     </row>
     <row r="37" spans="2:16" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B37" s="6" t="s">
@@ -1100,32 +1102,26 @@
       </c>
     </row>
     <row r="40" spans="2:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B40" s="20" t="s">
+      <c r="B40" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="20"/>
-      <c r="P40" s="20"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="11"/>
+      <c r="K40" s="11"/>
+      <c r="L40" s="11"/>
+      <c r="M40" s="11"/>
+      <c r="N40" s="11"/>
+      <c r="O40" s="11"/>
+      <c r="P40" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B3:F7"/>
-    <mergeCell ref="B13:M14"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B10:J11"/>
     <mergeCell ref="B40:P40"/>
     <mergeCell ref="B16:G17"/>
     <mergeCell ref="H16:I17"/>
@@ -1139,6 +1135,12 @@
     <mergeCell ref="H21:I23"/>
     <mergeCell ref="B33:L34"/>
     <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B3:F7"/>
+    <mergeCell ref="B13:M14"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B10:J11"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="74" fitToHeight="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="1200" r:id="rId1"/>

</xml_diff>